<commit_message>
updating sample batch upload filr for revesals
</commit_message>
<xml_diff>
--- a/public/files/sample_batch_linked_account_reversals.xlsx
+++ b/public/files/sample_batch_linked_account_reversals.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Transfer Id</t>
   </si>
@@ -19,13 +19,7 @@
     <t>Amount (In Paise)</t>
   </si>
   <si>
-    <t>notes</t>
-  </si>
-  <si>
     <t>trf_CKLJTXcMiGTGq2</t>
-  </si>
-  <si>
-    <t>Avinash: "asdf"</t>
   </si>
 </sst>
 </file>
@@ -105,19 +99,13 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1">
         <v>100.0</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding notes la refunds sample file
</commit_message>
<xml_diff>
--- a/public/files/sample_batch_linked_account_reversals.xlsx
+++ b/public/files/sample_batch_linked_account_reversals.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="6">
   <si>
     <t>Transfer Id</t>
   </si>
@@ -19,14 +19,23 @@
     <t>Amount (In Paise)</t>
   </si>
   <si>
+    <t>notes[1]</t>
+  </si>
+  <si>
+    <t>notes[2]</t>
+  </si>
+  <si>
     <t>trf_CKLJTXcMiGTGq2</t>
+  </si>
+  <si>
+    <t>note</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -34,8 +43,17 @@
     </font>
     <font/>
     <font>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <sz val="8.0"/>
       <color rgb="FF222222"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FF212121"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -59,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -68,6 +86,12 @@
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -99,13 +123,31 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
+      <c r="A2" s="3" t="s">
+        <v>4</v>
       </c>
       <c r="B2" s="1">
         <v>100.0</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix third notes coloum
</commit_message>
<xml_diff>
--- a/public/files/sample_batch_linked_account_reversals.xlsx
+++ b/public/files/sample_batch_linked_account_reversals.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
   <si>
     <t>Transfer Id</t>
   </si>
@@ -25,6 +25,9 @@
     <t>notes[2]</t>
   </si>
   <si>
+    <t>notes[3]</t>
+  </si>
+  <si>
     <t>trf_CKLJTXcMiGTGq2</t>
   </si>
   <si>
@@ -35,17 +38,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font/>
-    <font>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-    </font>
     <font>
       <sz val="8.0"/>
       <color rgb="FF222222"/>
@@ -77,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -87,10 +86,7 @@
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -129,25 +125,25 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>3</v>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
-        <v>4</v>
+      <c r="A2" s="2" t="s">
+        <v>5</v>
       </c>
       <c r="B2" s="1">
         <v>100.0</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>5</v>
+      <c r="C2" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>